<commit_message>
Update security review, handover and roadmap for authentication
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/FDE-Roadmap.xlsx
+++ b/docs/FDE-Roadmap.xlsx
@@ -1168,7 +1168,7 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>docs/05-test-strategy-and-results.md: 75 automated checks (29 Java, 25 Python, 19 console, 2 e2e) + 16-scenario agent eval, all green on H2. Honest gaps G1-G7: no Oracle run, no contract tests, no production-volume load test (no k6), no CDC, no real LLM, CI never run, no concurrency test.</t>
+          <t>docs/05: 34 Java, 27 Python, 23 console, 3 e2e (Edge) + 16-scenario agent eval, all green on H2. Authentication added: Basic auth, roles OPERATOR/REVIEWER/APPROVER/READER, actor from login, SWITCHED needs APPROVER, no default DB password, agent uses READER service account (docs/06 S1, S2 closed in code). Lesson: a 401 with WWW-Authenticate makes browsers hang on fetch, so the API sends a bare 401 and the console verifies credentials at sign-in. Gaps: no Oracle run, no contract tests, no k6 load test, no CDC, no real LLM (Zscaler), no concurrency test.</t>
         </is>
       </c>
     </row>
@@ -2246,7 +2246,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Partially: tested controls (PII-free prompts, no RAW_PAYLOAD in API, approval gates, audit, parameterised SQL) plus written review docs/06 with findings S1-S9. Biggest gap: no authn/z, approver is free text. Tenant isolation relies on TENANT_ID filters and has no cross-tenant test.</t>
+          <t>Partially: authentication and roles built and tested (SecurityApiTest, e2e wrong-password), secrets from env with no defaults, PII-free prompts, no RAW_PAYLOAD in API, approval gates, audit, parameterised SQL; review docs/06 (S1, S2 closed in code). Still open: OIDC/JWT for production and a cross-tenant isolation test.</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Update test results, signoff checklist and roadmap notes
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/FDE-Roadmap.xlsx
+++ b/docs/FDE-Roadmap.xlsx
@@ -1207,7 +1207,7 @@
       <c r="H18" s="2" t="inlineStr"/>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>docs/06-security-review.md: controls proven by tests (read-only agent, PII-free LLM prompts, no raw rows in API, parameterised SQL, approval gates, audit). Findings S1-S9: S1 no authn/z (approver is typed text) and S2 default DB password block real data. Fixes not yet applied.</t>
+          <t>docs/06-security-review.md: controls proven by tests (read-only agent, PII-free LLM prompts, no raw rows in API, parameterised SQL, approval gates, audit). Findings S1-S9: S1 no authn/z (approver is typed text) and S2 default DB password block real data. Fixes not yet applied. Update: checklist now 13 items; CI green on GitHub (G6 closed); demo script docs/08; repo public at github.com/JeswinSolomon/migration-orchestrator.</t>
         </is>
       </c>
     </row>
@@ -2250,7 +2250,11 @@
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
-      <c r="I26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>STAR: Situation: approvals were a typed name, so nobody could be held accountable. Task: add real authn/z fast without a customer IdP. Action: stateless Basic auth, 4 roles, actor taken from the login (request-body names ignored), env-only secrets, READER service account for the agent, cross-tenant tests. Result: S1/S2 closed in code; found that a 401 with WWW-Authenticate hangs browser fetch (headless e2e caught it), so the API returns a bare 401 and the UI verifies at sign-in. Next: OIDC/JWT.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -2320,7 +2324,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Done (docs): COO status update, failure-update template, signoff checklist with honest open items in docs/07. Interview angle: say what is proven, what is not, what you need from the customer, and do not promise a date before the Oracle rehearsal.</t>
+          <t>Done (docs): COO status update, failure-update template, signoff checklist with honest open items in docs/07. Interview angle: say what is proven, what is not, what you need from the customer, and do not promise a date before the Oracle rehearsal. Final pack: docs/07 signoff checklist (13 items, CI green on GitHub, 89 automated checks) and docs/08-demo-script.md. Demo-ready, not production-ready.</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Add concurrency and API contract tests; sync OpenAPI with real endpoints; update results
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/FDE-Roadmap.xlsx
+++ b/docs/FDE-Roadmap.xlsx
@@ -1168,7 +1168,7 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>docs/05: 34 Java, 27 Python, 23 console, 3 e2e (Edge) + 16-scenario agent eval, all green on H2. Authentication added: Basic auth, roles OPERATOR/REVIEWER/APPROVER/READER, actor from login, SWITCHED needs APPROVER, no default DB password, agent uses READER service account (docs/06 S1, S2 closed in code). Lesson: a 401 with WWW-Authenticate makes browsers hang on fetch, so the API sends a bare 401 and the console verifies credentials at sign-in. Gaps: no Oracle run, no contract tests, no k6 load test, no CDC, no real LLM (Zscaler), no concurrency test.</t>
+          <t>docs/05: 38 Java, 27 Python, 23 console, 3 e2e (91 total) (Edge) + 16-scenario agent eval, all green on H2. Authentication added: Basic auth, roles OPERATOR/REVIEWER/APPROVER/READER, actor from login, SWITCHED needs APPROVER, no default DB password, agent uses READER service account (docs/06 S1, S2 closed in code). Lesson: a 401 with WWW-Authenticate makes browsers hang on fetch, so the API sends a bare 401 and the console verifies credentials at sign-in. Gaps: no Oracle run, no contract tests, no k6 load test, no CDC, no real LLM (Zscaler), no concurrency test. Added: ConcurrentTransitionTest (6 racing callers, 1 winner, 5 x 409) and ApiContractTest (code vs OpenAPI endpoints; found 6 undocumented endpoints). G2 partly and G7 closed.</t>
         </is>
       </c>
     </row>
@@ -1913,7 +1913,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Partially: AI-client retry with exponential backoff, 4xx not retried, then 502 (HttpAiClientRetryTest); restartable per-batch transactions. DLQ and backpressure need Kafka (blocked). Interview angle: retry only idempotent/transient failures; cap attempts; always surface the final error.</t>
+          <t>Partially: AI-client retry with exponential backoff, 4xx not retried, then 502 (HttpAiClientRetryTest); restartable per-batch transactions. DLQ and backpressure need Kafka (blocked). Interview angle: retry only idempotent/transient failures; cap attempts; always surface the final error. Also proven: concurrent transition race gives exactly one winner (optimistic UPDATE ... WHERE STATE=?), others get 409.</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Add console data profile panel; update test counts and roadmap
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/FDE-Roadmap.xlsx
+++ b/docs/FDE-Roadmap.xlsx
@@ -1168,7 +1168,7 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>docs/05: 38 Java, 27 Python, 23 console, 3 e2e (91 total) (Edge) + 16-scenario agent eval, all green on H2. Authentication added: Basic auth, roles OPERATOR/REVIEWER/APPROVER/READER, actor from login, SWITCHED needs APPROVER, no default DB password, agent uses READER service account (docs/06 S1, S2 closed in code). Lesson: a 401 with WWW-Authenticate makes browsers hang on fetch, so the API sends a bare 401 and the console verifies credentials at sign-in. Gaps: no Oracle run, no contract tests, no k6 load test, no CDC, no real LLM (Zscaler), no concurrency test. Added: ConcurrentTransitionTest (6 racing callers, 1 winner, 5 x 409) and ApiContractTest (code vs OpenAPI endpoints; found 6 undocumented endpoints). G2 partly and G7 closed.</t>
+          <t>docs/05: 39 Java, 27 Python, 23 console, 3 e2e (94 total) (Edge) + 16-scenario agent eval, all green on H2. Authentication added: Basic auth, roles OPERATOR/REVIEWER/APPROVER/READER, actor from login, SWITCHED needs APPROVER, no default DB password, agent uses READER service account (docs/06 S1, S2 closed in code). Lesson: a 401 with WWW-Authenticate makes browsers hang on fetch, so the API sends a bare 401 and the console verifies credentials at sign-in. Gaps: no Oracle run, no contract tests, no k6 load test, no CDC, no real LLM (Zscaler), no concurrency test. Added: ConcurrentTransitionTest (6 racing callers, 1 winner, 5 x 409) and ApiContractTest (code vs OpenAPI endpoints; found 6 undocumented endpoints). G2 partly and G7 closed.</t>
         </is>
       </c>
     </row>
@@ -1207,7 +1207,7 @@
       <c r="H18" s="2" t="inlineStr"/>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>docs/06-security-review.md: controls proven by tests (read-only agent, PII-free LLM prompts, no raw rows in API, parameterised SQL, approval gates, audit). Findings S1-S9: S1 no authn/z (approver is typed text) and S2 default DB password block real data. Fixes not yet applied. Update: checklist now 13 items; CI green on GitHub (G6 closed); demo script docs/08; repo public at github.com/jeswinstaynes01-dev/migration-orchestrator.</t>
+          <t>docs/06-security-review.md: controls proven by tests (read-only agent, PII-free LLM prompts, no raw rows in API, parameterised SQL, approval gates, audit). Findings S1-S9: S1 no authn/z (approver is typed text) and S2 default DB password block real data. Fixes not yet applied. Update: checklist now 13 items; CI green on GitHub (G6 closed); demo script docs/08; repo public at github.com/jeswinstaynes01-dev/migration-orchestrator. FR1 data profiling now built: GET /api/runs/{id}/profile (null rates, duplicates, date-format mix, counts only so PII-free) plus console Data profile panel; tests ProfileServiceTest and ProfilePanel.test.</t>
         </is>
       </c>
     </row>
@@ -1399,7 +1399,11 @@
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Update: profiling is now an API (/api/runs/{id}/profile) and a console panel; reports counts only (no raw values) so it is PII-free; tested by ProfileServiceTest.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">

</xml_diff>

<commit_message>
Add Pending & Dependencies sheet to the roadmap
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/FDE-Roadmap.xlsx
+++ b/docs/FDE-Roadmap.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Learning Trace" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending &amp; Dependencies" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -65,7 +66,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -74,6 +75,9 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2514,4 +2518,414 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Pending item</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Blocked by</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>What is needed to finish</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>Current workaround / what is proven</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Run against real Oracle target</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Goal G1/G2, FR3, FR6</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Docker not installed</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Install</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Docker Desktop, Oracle XE container, point TARGET_DB_URL at it, rerun the test suite and load</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>All logic proven on H2 in Oracle mode (66k-row run, reconciliation ties out)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>CDC via Kafka and Debezium, final sync</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>FR4, FR9, NFR lag p95 &lt; 5 s</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Docker not installed</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Install</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Docker Compose with PostgreSQL, Kafka, Debezium; build the consumer and final-sync step</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Event contract in docs/contracts/kafka-events.md; state machine and pre-checks already gate FINAL_SYNC</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>PostgreSQL as the legacy source</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Decision 1 in docs/01</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Docker not installed</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Install</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>PostgreSQL container and a source reader</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Legacy data is read from CSV files</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Real LLM for mapping and diagnosis quality</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Goal G4 (measured on a real model)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Corporate web filter (Zscaler) blocks model download</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Access / IT</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Allow registry.ollama.ai or provide a hosted OpenAI-compatible endpoint and key</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Rule-based agent scores 16/16 on evals; HTTP LLM path tested against a fake server; Ollama is installed</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>OIDC/JWT single sign-on</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>NFR role-based access</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Needs an identity provider</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Access / IT</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>IdP details (issuer, client), swap Basic auth for resource-server JWT</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Basic auth, 4 roles, actor from login, tested</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Throughput proof (&gt;= 5k rows/s) and CDC lag</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>NFR throughput</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Needs Oracle and a production-size run</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Install</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Run the 400k-loan / 6M-payment load on the real target</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>66k rows measured on H2 only</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>DLQ and replay view in the console</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>FR9, FR11</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Depends on item 2 (no DLQ exists without Kafka)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Build after item 2</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>DLQ API plus console panel</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Exceptions (quarantined rows), reconciliation, profile, diagnose panels exist</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Agent chat and traces/alerts</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>FR11, NFR observability</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Time; traces need a collector (install)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Build / Install</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Chat UI, OpenTelemetry collector, alert rules</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Metrics (Micrometer) and a single-question diagnose panel</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Body-schema contract tests, PII masking check in logs</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>NFR security, G2</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Time only</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Validate bodies against OpenAPI; scan logs for PII</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Endpoint-level contract test; PII-free prompts and API</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Customer approver and negative-amount owner named; sign-off names and dates</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>docs/07 checklist item 10</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Needs the business</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Names from the customer</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Open items listed in docs/07</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>